<commit_message>
docs(sync): update testing workbooks with 34 tests and reconcile notifyUser coverage documentation
</commit_message>
<xml_diff>
--- a/deliverables/i243164_i243137_i243088_SE_C.xlsx
+++ b/deliverables/i243164_i243137_i243088_SE_C.xlsx
@@ -432,7 +432,7 @@
     <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
     <ns0:pageSetUpPr/>
   </ns0:sheetPr>
-  <ns0:dimension ref="A1:H28"/>
+  <ns0:dimension ref="A1:H35"/>
   <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <ns0:cols>
     <ns0:col width="22" customWidth="1" min="1" max="1"/>
@@ -1618,6 +1618,300 @@
       <ns0:c r="H28" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t>design/test_designs.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-28</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::updateParams</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Reload COM_FAIL_ACT_T delay parameter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Modify COM_FAIL_ACT_T to 7.5s, call updateParams()</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Internal action delay updated to 7.5s</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:143-147, framework.h:297</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1377</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30">
+      <ns0:c r="A30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-29</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::removeAction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Action removal and duplicate caller diagnostic</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Cleared failure transition; duplicate action injection</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Action removed; duplicate diagnostic logged</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:376-388</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1400</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-30</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::getSelectedAction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mode fallback cascade (PosCtrl-&gt;AltCtrl-&gt;Stab)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Cascade degraded sensor requirements for each fallback</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Orderly fallback PosCtrl -&gt; AltCtrl -&gt; Stab -&gt; Terminate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:540-564</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1442</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-31</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::getSelectedAction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Redundant UX warning guards (RTL/Land/Precland)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Active and unavailable combinations for RTL &amp; Land</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Suppresses repeated action; issues Warn notification</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:619-644</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1498</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-32</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::deferFailsafes</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Deferral edge cases (active action, disable, timeout=0)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Active serious action; enable/disable; timeout=0</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Returns false on serious action; delay resets; default timeout</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:721-729</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1539</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34">
+      <ns0:c r="A34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-33</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::checkFailsafe</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Individual decision branch coverage (slots, takeover)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Slot index allocation, takeover thresholds, caller checks</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>All individual decision branches reached</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:320, 401, 409, 426, 483, 495, 508</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1579</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="35">
+      <ns0:c r="A35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TC-FS-34</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FailsafeBase::notifyUser</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Full notification branch coverage (actions, causes)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Delayed/immediate actions; specific battery &amp; link causes</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>All notification branches dispatched</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>framework.cpp:185-298</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>failsafe_student_test.cpp:1625</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>

</xml_diff>